<commit_message>
data: release 2.0, two rows that point to no data removed
</commit_message>
<xml_diff>
--- a/DATABASE.xlsx
+++ b/DATABASE.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V323"/>
+  <dimension ref="A1:V321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21716,7 +21716,7 @@
     </row>
     <row r="270">
       <c r="A270" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B270" t="inlineStr">
         <is>
@@ -21725,58 +21725,86 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Genetically Predicted Social Connections And Risk Of Cognitive Impairment: A Mendelian Randomization Study.</t>
+          <t>The Role Of Country-Level Characteristics For The Association Between Loneliness And Neighborhood Cohesion - A Multi-Level Analysis</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.jad.2024.08.106</t>
+          <t>https://doi.org/10.1177/02654075241262321</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Genome-Wide Association Study</t>
+          <t>European Social Survey - ESS6 - 2012</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>GWAS</t>
-        </is>
+          <t>ESS</t>
+        </is>
+      </c>
+      <c r="G270" t="n">
+        <v>2012</v>
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>https://www.sciencedirect.com/topics/agricultural-and-biological-sciences/genome-wide-association-study</t>
+          <t>https://ess.sikt.no/en/</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Austria, Belgium, Czech Republic, Finland, France, Germany, Hungary, Ireland, Italy, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Estonia, Spain, United Kingdom, Lithuania</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t>Cross-section</t>
+          <t>Repeated cross-section</t>
+        </is>
+      </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="N270" t="inlineStr">
+        <is>
+          <t>Adults</t>
+        </is>
+      </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="P270" t="inlineStr">
+        <is>
+          <t>you felt lonely?</t>
         </is>
       </c>
       <c r="S270" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U270" t="inlineStr">
-        <is>
-          <t>This is just a commentary to this paper: https://www.sciencedirect.com/science/article/pii/S0165032724000193?via%3Dihub</t>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="T270" t="inlineStr">
+        <is>
+          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Media use</t>
         </is>
       </c>
       <c r="V270" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B271" t="inlineStr">
         <is>
@@ -21785,22 +21813,22 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>The Role Of Country-Level Characteristics For The Association Between Loneliness And Neighborhood Cohesion - A Multi-Level Analysis</t>
+          <t>Early-Life Circumstances And Late Life Loneliness Trajectories Among Finnish Older Adults</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/02654075241262321</t>
+          <t>https://doi.org/10.1186/s12877-024-04967-6</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>European Social Survey - ESS6 - 2012</t>
+          <t>Good Ageing in Lahti region - GOAL</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>ESS</t>
+          <t>GOAL</t>
         </is>
       </c>
       <c r="G271" t="n">
@@ -21808,22 +21836,25 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>https://ess.sikt.no/en/</t>
+          <t>https://blogs.helsinki.fi/ikihyva-paijat-hame/in-english-2/</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Czech Republic, Finland, France, Germany, Hungary, Ireland, Italy, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Estonia, Spain, United Kingdom, Lithuania</t>
-        </is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="J271" t="n">
+        <v>1552</v>
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>CAWI</t>
         </is>
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>Repeated cross-section</t>
+          <t>Panel</t>
         </is>
       </c>
       <c r="M271" t="inlineStr">
@@ -21833,17 +21864,22 @@
       </c>
       <c r="N271" t="inlineStr">
         <is>
-          <t>Adults</t>
-        </is>
-      </c>
-      <c r="O271" t="inlineStr">
-        <is>
-          <t>D9</t>
+          <t>Old</t>
         </is>
       </c>
       <c r="P271" t="inlineStr">
         <is>
-          <t>you felt lonely?</t>
+          <t>Do you feel lonely?</t>
+        </is>
+      </c>
+      <c r="Q271" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R271" t="inlineStr">
+        <is>
+          <t>Never-All the time</t>
         </is>
       </c>
       <c r="S271" t="inlineStr">
@@ -21851,20 +21887,20 @@
           <t>Direct</t>
         </is>
       </c>
-      <c r="T271" t="inlineStr">
-        <is>
-          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Media use</t>
+      <c r="U271" t="inlineStr">
+        <is>
+          <t>Impossible to retrieve codebook of the survey</t>
         </is>
       </c>
       <c r="V271" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="n">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B272" t="inlineStr">
         <is>
@@ -21873,39 +21909,36 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Early-Life Circumstances And Late Life Loneliness Trajectories Among Finnish Older Adults</t>
+          <t>Gender And Socioeconomic Perspectives On Students' Emotional Well-Being During The Covid-19 Pandemic</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1186/s12877-024-04967-6</t>
+          <t>https://doi.org/10.1177/17454999241265966</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Good Ageing in Lahti region - GOAL</t>
+          <t>Responses to Educational Disruption Survey - REDS</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>GOAL</t>
-        </is>
-      </c>
-      <c r="G272" t="n">
-        <v>2012</v>
+          <t>REDS</t>
+        </is>
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>https://blogs.helsinki.fi/ikihyva-paijat-hame/in-english-2/</t>
+          <t>https://www.iea.nl/studies/iea/REDS</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="J272" t="n">
-        <v>1552</v>
+        <v>13398</v>
       </c>
       <c r="K272" t="inlineStr">
         <is>
@@ -21914,7 +21947,7 @@
       </c>
       <c r="L272" t="inlineStr">
         <is>
-          <t>Panel</t>
+          <t>Cross-section</t>
         </is>
       </c>
       <c r="M272" t="inlineStr">
@@ -21924,22 +21957,12 @@
       </c>
       <c r="N272" t="inlineStr">
         <is>
-          <t>Old</t>
+          <t>Young</t>
         </is>
       </c>
       <c r="P272" t="inlineStr">
         <is>
-          <t>Do you feel lonely?</t>
-        </is>
-      </c>
-      <c r="Q272" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="R272" t="inlineStr">
-        <is>
-          <t>Never-All the time</t>
+          <t>I felt more lonely than usual</t>
         </is>
       </c>
       <c r="S272" t="inlineStr">
@@ -21960,7 +21983,7 @@
     </row>
     <row r="273">
       <c r="A273" t="n">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B273" t="inlineStr">
         <is>
@@ -21969,38 +21992,48 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>The Societal Cost Of 'Unwanted' Loneliness In Spain</t>
+          <t>The Role Of Social Network Structure And Function In Moderate And Severe Social And Emotional Loneliness: The Dutch SaNAE Study In Older Adults</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s10198-024-01724-9</t>
+          <t>https://doi.org/10.1016/j.heliyon.2023.e23734</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>Private data</t>
+          <t>SaNAE cohort</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>SaNAE</t>
         </is>
       </c>
       <c r="G273" t="n">
-        <v>2022</v>
+        <v>2020</v>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>https://www.ggdzl.nl/professionals/projecten-en-onderzoeken/sanae/</t>
+        </is>
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="J273" t="n">
-        <v>4004</v>
+        <v>3396</v>
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>CATI</t>
+          <t>CAWI</t>
         </is>
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t>Cross-section</t>
+          <t>Repeated cross-section</t>
         </is>
       </c>
       <c r="M273" t="inlineStr">
@@ -22010,32 +22043,37 @@
       </c>
       <c r="N273" t="inlineStr">
         <is>
-          <t>Adults</t>
+          <t>Old</t>
+        </is>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t xml:space="preserve">; ; ; ; ; </t>
         </is>
       </c>
       <c r="P273" t="inlineStr">
         <is>
-          <t>Regardless of how much or how little contact you have with other people in your daily life, how often do you feel lonely? By feeling lonely we mean that you have fewer relationships with other people than you would like, or the relationships you do have do not offer you as much support as you would like</t>
+          <t>There are plenty of people I can rely on when I have problems; There are many people whom I can trust completely; There are enough people I feel close to; I experience a general sense of emptiness; I miss having people around; I often feel rejected</t>
         </is>
       </c>
       <c r="Q273" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5; 5; 5; 5; 5; 5</t>
         </is>
       </c>
       <c r="R273" t="inlineStr">
         <is>
-          <t>Never-Always</t>
+          <t>totally agree - totally disagree; totally agree - totally disagree; totally agree - totally disagree; totally agree - totally disagree; totally agree - totally disagree; totally agree - totally disagree</t>
         </is>
       </c>
       <c r="S273" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>DJG-6</t>
         </is>
       </c>
       <c r="U273" t="inlineStr">
         <is>
-          <t>Impossible to retrieve codebook of the survey</t>
+          <t>Item wording from the published study: https://pmc.ncbi.nlm.nih.gov/articles/PMC10788429/</t>
         </is>
       </c>
       <c r="V273" t="inlineStr">
@@ -22046,7 +22084,7 @@
     </row>
     <row r="274">
       <c r="A274" t="n">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B274" t="inlineStr">
         <is>
@@ -22055,36 +22093,39 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Gender And Socioeconomic Perspectives On Students' Emotional Well-Being During The Covid-19 Pandemic</t>
+          <t>Loneliness During The Covid-19 Pandemic: Evidence From Five European Countries</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/17454999241265966</t>
+          <t>https://doi.org/10.1016/j.ehb.2024.101427</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Responses to Educational Disruption Survey - REDS</t>
+          <t>COVID-19, MEntal HEalth, REsilience and SElf-regulation - COME-HERE</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>REDS</t>
-        </is>
+          <t>COME-HERE</t>
+        </is>
+      </c>
+      <c r="G274" t="n">
+        <v>2022</v>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>https://www.iea.nl/studies/iea/REDS</t>
+          <t>https://www.uni.lu/fhse-en/research-projects/pandemic-pandoras-box-the-demographic-economic-social-and-psychological-impact-of-covid19/pandemic-come-here-survey/</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>France, Germany, Italy, Spain, Sweden</t>
         </is>
       </c>
       <c r="J274" t="n">
-        <v>13398</v>
+        <v>11059</v>
       </c>
       <c r="K274" t="inlineStr">
         <is>
@@ -22093,7 +22134,7 @@
       </c>
       <c r="L274" t="inlineStr">
         <is>
-          <t>Cross-section</t>
+          <t>Panel</t>
         </is>
       </c>
       <c r="M274" t="inlineStr">
@@ -22103,22 +22144,32 @@
       </c>
       <c r="N274" t="inlineStr">
         <is>
-          <t>Young</t>
+          <t>Adults</t>
         </is>
       </c>
       <c r="P274" t="inlineStr">
         <is>
-          <t>I felt more lonely than usual</t>
+          <t>UCLA</t>
+        </is>
+      </c>
+      <c r="Q274" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R274" t="inlineStr">
+        <is>
+          <t>Hardly ever-Often</t>
         </is>
       </c>
       <c r="S274" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="U274" t="inlineStr">
         <is>
-          <t>Impossible to retrieve codebook of the survey</t>
+          <t>Impossible to retrieve codebook of the survey; UCLA-8</t>
         </is>
       </c>
       <c r="V274" t="inlineStr">
@@ -22129,7 +22180,7 @@
     </row>
     <row r="275">
       <c r="A275" t="n">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B275" t="inlineStr">
         <is>
@@ -22138,22 +22189,22 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>The Role Of Social Network Structure And Function In Moderate And Severe Social And Emotional Loneliness: The Dutch SaNAE Study In Older Adults</t>
+          <t>The Mediating Role Of Digital Competence In The Associations Between The Factors Affecting Healthcare Utilization And Access To Care.</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.heliyon.2023.e23734</t>
+          <t>https://doi.org/10.3389/ijph.2023.1606184</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>SaNAE cohort</t>
+          <t>FinHealth</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>SaNAE</t>
+          <t>FinHealth</t>
         </is>
       </c>
       <c r="G275" t="n">
@@ -22161,16 +22212,16 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>https://www.ggdzl.nl/professionals/projecten-en-onderzoeken/sanae/</t>
+          <t>https://thl.fi/en/research-and-development/research-and-projects/national-finhealth-study-</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="J275" t="n">
-        <v>3396</v>
+        <v>4881</v>
       </c>
       <c r="K275" t="inlineStr">
         <is>
@@ -22179,7 +22230,7 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>Repeated cross-section</t>
+          <t>Panel</t>
         </is>
       </c>
       <c r="M275" t="inlineStr">
@@ -22189,37 +22240,32 @@
       </c>
       <c r="N275" t="inlineStr">
         <is>
-          <t>Old</t>
-        </is>
-      </c>
-      <c r="O275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">; ; ; ; ; </t>
+          <t>Adults</t>
         </is>
       </c>
       <c r="P275" t="inlineStr">
         <is>
-          <t>There are plenty of people I can rely on when I have problems; There are many people whom I can trust completely; There are enough people I feel close to; I experience a general sense of emptiness; I miss having people around; I often feel rejected</t>
+          <t>Do you ever feel lonely?</t>
         </is>
       </c>
       <c r="Q275" t="inlineStr">
         <is>
-          <t>5; 5; 5; 5; 5; 5</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R275" t="inlineStr">
         <is>
-          <t>totally agree - totally disagree; totally agree - totally disagree; totally agree - totally disagree; totally agree - totally disagree; totally agree - totally disagree; totally agree - totally disagree</t>
+          <t>Never-All the time</t>
         </is>
       </c>
       <c r="S275" t="inlineStr">
         <is>
-          <t>DJG-6</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="U275" t="inlineStr">
         <is>
-          <t>Item wording from the published study: https://pmc.ncbi.nlm.nih.gov/articles/PMC10788429/</t>
+          <t>Item wording from the published study: https://doi.org/10.3389/ijph.2023.1606184</t>
         </is>
       </c>
       <c r="V275" t="inlineStr">
@@ -22230,7 +22276,7 @@
     </row>
     <row r="276">
       <c r="A276" t="n">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B276" t="inlineStr">
         <is>
@@ -22239,39 +22285,34 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Loneliness During The Covid-19 Pandemic: Evidence From Five European Countries</t>
+          <t>Long-Term Sequelae Of Sars-Cov-2 Two Years Following Infection: Exploring The Interplay Of Biological, Psychological, And Social Factors.</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.ehb.2024.101427</t>
+          <t>https://doi.org/10.1017/S0033291724002721</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>COVID-19, MEntal HEalth, REsilience and SElf-regulation - COME-HERE</t>
+          <t>RECoVERED</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>COME-HERE</t>
+          <t>RECoVERED</t>
         </is>
       </c>
       <c r="G276" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H276" t="inlineStr">
-        <is>
-          <t>https://www.uni.lu/fhse-en/research-projects/pandemic-pandoras-box-the-demographic-economic-social-and-psychological-impact-of-covid19/pandemic-come-here-survey/</t>
-        </is>
+        <v>2021</v>
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>France, Germany, Italy, Spain, Sweden</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="J276" t="n">
-        <v>11059</v>
+        <v>68</v>
       </c>
       <c r="K276" t="inlineStr">
         <is>
@@ -22285,17 +22326,17 @@
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>Representative</t>
+          <t>Convenience</t>
         </is>
       </c>
       <c r="N276" t="inlineStr">
         <is>
-          <t>Adults</t>
+          <t>Clinical</t>
         </is>
       </c>
       <c r="P276" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>DJG-6</t>
         </is>
       </c>
       <c r="Q276" t="inlineStr">
@@ -22305,17 +22346,17 @@
       </c>
       <c r="R276" t="inlineStr">
         <is>
-          <t>Hardly ever-Often</t>
+          <t>Yes-No</t>
         </is>
       </c>
       <c r="S276" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>DJG-6</t>
         </is>
       </c>
       <c r="U276" t="inlineStr">
         <is>
-          <t>Impossible to retrieve codebook of the survey; UCLA-8</t>
+          <t>Impossible to retrieve codebook of the survey</t>
         </is>
       </c>
       <c r="V276" t="inlineStr">
@@ -22326,7 +22367,7 @@
     </row>
     <row r="277">
       <c r="A277" t="n">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B277" t="inlineStr">
         <is>
@@ -22335,22 +22376,22 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>The Mediating Role Of Digital Competence In The Associations Between The Factors Affecting Healthcare Utilization And Access To Care.</t>
+          <t>A Machine Learning Approach To Identifying Risk Factors For Long Covid-19</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3389/ijph.2023.1606184</t>
+          <t>https://doi.org/10.3390/a17110485</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>FinHealth</t>
+          <t>Understanding Society: COVID-19 Study- April 2020</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>FinHealth</t>
+          <t>USC</t>
         </is>
       </c>
       <c r="G277" t="n">
@@ -22358,20 +22399,17 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>https://thl.fi/en/research-and-development/research-and-projects/national-finhealth-study-</t>
+          <t>https://datacatalogue.ukdataservice.ac.uk/studies/study/8644#details</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
         <is>
-          <t>Finland</t>
-        </is>
-      </c>
-      <c r="J277" t="n">
-        <v>4881</v>
+          <t>United Kingdom</t>
+        </is>
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t>CAWI</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="L277" t="inlineStr">
@@ -22389,19 +22427,24 @@
           <t>Adults</t>
         </is>
       </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>sclonely_cv</t>
+        </is>
+      </c>
       <c r="P277" t="inlineStr">
         <is>
-          <t>Do you ever feel lonely?</t>
+          <t>In the last 4 weeks, how often did you feel lonely?</t>
         </is>
       </c>
       <c r="Q277" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R277" t="inlineStr">
         <is>
-          <t>Never-All the time</t>
+          <t>Hardly ever or never - Often</t>
         </is>
       </c>
       <c r="S277" t="inlineStr">
@@ -22409,20 +22452,20 @@
           <t>Direct</t>
         </is>
       </c>
-      <c r="U277" t="inlineStr">
-        <is>
-          <t>Item wording from the published study: https://doi.org/10.3389/ijph.2023.1606184</t>
+      <c r="T277" t="inlineStr">
+        <is>
+          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Care and welfare use, COVID-19, Online activities</t>
         </is>
       </c>
       <c r="V277" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="n">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B278" t="inlineStr">
         <is>
@@ -22431,38 +22474,40 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Long-Term Sequelae Of Sars-Cov-2 Two Years Following Infection: Exploring The Interplay Of Biological, Psychological, And Social Factors.</t>
+          <t>A Machine Learning Approach To Identifying Risk Factors For Long Covid-19</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1017/S0033291724002721</t>
+          <t>https://doi.org/10.3390/a17110485</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>RECoVERED</t>
+          <t>Understanding Society: COVID-19 Study- May 2020</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>RECoVERED</t>
+          <t>USC</t>
         </is>
       </c>
       <c r="G278" t="n">
-        <v>2021</v>
+        <v>2020</v>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>https://datacatalogue.ukdataservice.ac.uk/studies/study/8644#details</t>
+        </is>
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
-      <c r="J278" t="n">
-        <v>68</v>
+          <t>United Kingdom</t>
+        </is>
       </c>
       <c r="K278" t="inlineStr">
         <is>
-          <t>CAWI</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="L278" t="inlineStr">
@@ -22472,17 +22517,22 @@
       </c>
       <c r="M278" t="inlineStr">
         <is>
-          <t>Convenience</t>
+          <t>Representative</t>
         </is>
       </c>
       <c r="N278" t="inlineStr">
         <is>
-          <t>Clinical</t>
+          <t>Adults</t>
+        </is>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>sclonely_cv</t>
         </is>
       </c>
       <c r="P278" t="inlineStr">
         <is>
-          <t>DJG-6</t>
+          <t>In the last 4 weeks, how often did you feel lonely?</t>
         </is>
       </c>
       <c r="Q278" t="inlineStr">
@@ -22492,28 +22542,28 @@
       </c>
       <c r="R278" t="inlineStr">
         <is>
-          <t>Yes-No</t>
+          <t>Hardly ever or never - Often</t>
         </is>
       </c>
       <c r="S278" t="inlineStr">
         <is>
-          <t>DJG-6</t>
-        </is>
-      </c>
-      <c r="U278" t="inlineStr">
-        <is>
-          <t>Impossible to retrieve codebook of the survey</t>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="T278" t="inlineStr">
+        <is>
+          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Care and welfare use, COVID-19, Online activities</t>
         </is>
       </c>
       <c r="V278" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B279" t="inlineStr">
         <is>
@@ -22532,7 +22582,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Understanding Society: COVID-19 Study- April 2020</t>
+          <t>Understanding Society: COVID-19 Study- June 2020</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -22611,7 +22661,7 @@
     </row>
     <row r="280">
       <c r="A280" t="n">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B280" t="inlineStr">
         <is>
@@ -22630,7 +22680,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Understanding Society: COVID-19 Study- May 2020</t>
+          <t>Understanding Society: COVID-19 Study- July 2020</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -22709,7 +22759,7 @@
     </row>
     <row r="281">
       <c r="A281" t="n">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B281" t="inlineStr">
         <is>
@@ -22728,7 +22778,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Understanding Society: COVID-19 Study- June 2020</t>
+          <t>Understanding Society: COVID-19 Study- September 2020</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
@@ -22807,7 +22857,7 @@
     </row>
     <row r="282">
       <c r="A282" t="n">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B282" t="inlineStr">
         <is>
@@ -22826,7 +22876,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Understanding Society: COVID-19 Study- July 2020</t>
+          <t>Understanding Society: COVID-19 Study- November 2020</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -22905,7 +22955,7 @@
     </row>
     <row r="283">
       <c r="A283" t="n">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B283" t="inlineStr">
         <is>
@@ -22924,7 +22974,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Understanding Society: COVID-19 Study- September 2020</t>
+          <t>Understanding Society: COVID-19 Study- January 2021</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -22933,7 +22983,7 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="H283" t="inlineStr">
         <is>
@@ -23003,7 +23053,7 @@
     </row>
     <row r="284">
       <c r="A284" t="n">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B284" t="inlineStr">
         <is>
@@ -23022,7 +23072,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Understanding Society: COVID-19 Study- November 2020</t>
+          <t>Understanding Society: COVID-19 Study- March 2021</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -23031,7 +23081,7 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
@@ -23101,7 +23151,7 @@
     </row>
     <row r="285">
       <c r="A285" t="n">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B285" t="inlineStr">
         <is>
@@ -23120,7 +23170,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Understanding Society: COVID-19 Study- January 2021</t>
+          <t>Understanding Society: COVID-19 Study- September 2021</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
@@ -23199,7 +23249,7 @@
     </row>
     <row r="286">
       <c r="A286" t="n">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B286" t="inlineStr">
         <is>
@@ -23208,40 +23258,43 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>A Machine Learning Approach To Identifying Risk Factors For Long Covid-19</t>
+          <t>Development Of Nature-Related Habits And Their Relation To Mental Health Outcomes During Two Years Of The Covid-19 Pandemic: A Population-Based Study In Sweden</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/a17110485</t>
+          <t>https://doi.org/10.1007/s10389-024-02230-1</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Understanding Society: COVID-19 Study- March 2021</t>
+          <t>Swedish Longitudinal Occupational Survey of Health - SLOSH</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>USC</t>
+          <t>SLOSH</t>
         </is>
       </c>
       <c r="G286" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>https://datacatalogue.ukdataservice.ac.uk/studies/study/8644#details</t>
+          <t>https://slosh.se/for-researchers-in-english/introduction</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
-        </is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="J286" t="n">
+        <v>1580</v>
       </c>
       <c r="K286" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>CAWI</t>
         </is>
       </c>
       <c r="L286" t="inlineStr">
@@ -23259,14 +23312,9 @@
           <t>Adults</t>
         </is>
       </c>
-      <c r="O286" t="inlineStr">
-        <is>
-          <t>sclonely_cv</t>
-        </is>
-      </c>
       <c r="P286" t="inlineStr">
         <is>
-          <t>In the last 4 weeks, how often did you feel lonely?</t>
+          <t>UCLA-3</t>
         </is>
       </c>
       <c r="Q286" t="inlineStr">
@@ -23276,28 +23324,28 @@
       </c>
       <c r="R286" t="inlineStr">
         <is>
-          <t>Hardly ever or never - Often</t>
+          <t>Never-Often</t>
         </is>
       </c>
       <c r="S286" t="inlineStr">
         <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="T286" t="inlineStr">
-        <is>
-          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Care and welfare use, COVID-19, Online activities</t>
+          <t>UCLA-3</t>
+        </is>
+      </c>
+      <c r="U286" t="inlineStr">
+        <is>
+          <t>Impossible to retrieve codebook of the survey</t>
         </is>
       </c>
       <c r="V286" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="n">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B287" t="inlineStr">
         <is>
@@ -23306,65 +23354,60 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>A Machine Learning Approach To Identifying Risk Factors For Long Covid-19</t>
+          <t>Factors Associated With Health‐Related Quality Of Life Among Community‐Dwelling Older Adults: The APPCARE Study</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/a17110485</t>
+          <t>https://doi.org/10.1038/s41598-024-64539-x</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Understanding Society: COVID-19 Study- September 2021</t>
+          <t>Appropriate care paths for frail elderly people: a comprehensive model - APPCARE</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>USC</t>
-        </is>
-      </c>
-      <c r="G287" t="n">
-        <v>2021</v>
+          <t>APPCARE</t>
+        </is>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>https://datacatalogue.ukdataservice.ac.uk/studies/study/8644#details</t>
+          <t>https://kveloce.com/project/appcare-appropriate-care-paths-for-frail-elderly-patients-a-comprehensive-model/?lang=en</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
-        </is>
+          <t>Netherlands, Italy, Spain</t>
+        </is>
+      </c>
+      <c r="J287" t="n">
+        <v>865</v>
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>CAWI</t>
         </is>
       </c>
       <c r="L287" t="inlineStr">
         <is>
-          <t>Panel</t>
+          <t>Cross-section</t>
         </is>
       </c>
       <c r="M287" t="inlineStr">
         <is>
-          <t>Representative</t>
+          <t>Convenience</t>
         </is>
       </c>
       <c r="N287" t="inlineStr">
         <is>
-          <t>Adults</t>
-        </is>
-      </c>
-      <c r="O287" t="inlineStr">
-        <is>
-          <t>sclonely_cv</t>
+          <t>Old</t>
         </is>
       </c>
       <c r="P287" t="inlineStr">
         <is>
-          <t>In the last 4 weeks, how often did you feel lonely?</t>
+          <t>DJG-6</t>
         </is>
       </c>
       <c r="Q287" t="inlineStr">
@@ -23374,28 +23417,28 @@
       </c>
       <c r="R287" t="inlineStr">
         <is>
-          <t>Hardly ever or never - Often</t>
+          <t>Yes-No</t>
         </is>
       </c>
       <c r="S287" t="inlineStr">
         <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="T287" t="inlineStr">
-        <is>
-          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Care and welfare use, COVID-19, Online activities</t>
+          <t>DJG-6</t>
+        </is>
+      </c>
+      <c r="U287" t="inlineStr">
+        <is>
+          <t>Impossible to retrieve codebook of the survey</t>
         </is>
       </c>
       <c r="V287" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="n">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
@@ -23404,39 +23447,39 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Development Of Nature-Related Habits And Their Relation To Mental Health Outcomes During Two Years Of The Covid-19 Pandemic: A Population-Based Study In Sweden</t>
+          <t>General Self‐Efficacy, Not Musculoskeletal Health, Was Associated With Social Isolation And Loneliness In Older Adults During The Covid‐19 Pandemic: Findings From The Hertfordshire Cohort Study</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s10389-024-02230-1</t>
+          <t>https://doi.org/10.1007/s40520-023-02676-5</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Swedish Longitudinal Occupational Survey of Health - SLOSH</t>
+          <t>Hertfordshire Cohort Study</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>SLOSH</t>
+          <t>HCS</t>
         </is>
       </c>
       <c r="G288" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>https://slosh.se/for-researchers-in-english/introduction</t>
+          <t>https://www.mrc.soton.ac.uk/herts/</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="J288" t="n">
-        <v>1580</v>
+        <v>176</v>
       </c>
       <c r="K288" t="inlineStr">
         <is>
@@ -23450,17 +23493,17 @@
       </c>
       <c r="M288" t="inlineStr">
         <is>
-          <t>Representative</t>
+          <t>Convenience</t>
         </is>
       </c>
       <c r="N288" t="inlineStr">
         <is>
-          <t>Adults</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="P288" t="inlineStr">
         <is>
-          <t>UCLA-3</t>
+          <t>DJG-6</t>
         </is>
       </c>
       <c r="Q288" t="inlineStr">
@@ -23470,12 +23513,12 @@
       </c>
       <c r="R288" t="inlineStr">
         <is>
-          <t>Never-Often</t>
+          <t>Yes-No</t>
         </is>
       </c>
       <c r="S288" t="inlineStr">
         <is>
-          <t>UCLA-3</t>
+          <t>DJG-6</t>
         </is>
       </c>
       <c r="U288" t="inlineStr">
@@ -23491,7 +23534,7 @@
     </row>
     <row r="289">
       <c r="A289" t="n">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B289" t="inlineStr">
         <is>
@@ -23500,45 +23543,48 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Factors Associated With Health‐Related Quality Of Life Among Community‐Dwelling Older Adults: The APPCARE Study</t>
+          <t>Social Dysfunction And Neural Processing Of Emotional Valence Across Depressive And Anxiety Disorders</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1038/s41598-024-64539-x</t>
+          <t>https://doi.org/10.1155/2024/8564344</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Appropriate care paths for frail elderly people: a comprehensive model - APPCARE</t>
+          <t>Netherlands Study of Depression and Anxiety - NESDA</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>APPCARE</t>
-        </is>
+          <t>NSDA</t>
+        </is>
+      </c>
+      <c r="G289" t="n">
+        <v>2007</v>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>https://kveloce.com/project/appcare-appropriate-care-paths-for-frail-elderly-patients-a-comprehensive-model/?lang=en</t>
+          <t>https://onlinelibrary.wiley.com/doi/10.1002/mpr.256</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
         <is>
-          <t>Netherlands, Italy, Spain</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="J289" t="n">
-        <v>865</v>
+        <v>200</v>
       </c>
       <c r="K289" t="inlineStr">
         <is>
-          <t>CAWI</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="L289" t="inlineStr">
         <is>
-          <t>Cross-section</t>
+          <t>Panel</t>
         </is>
       </c>
       <c r="M289" t="inlineStr">
@@ -23548,7 +23594,7 @@
       </c>
       <c r="N289" t="inlineStr">
         <is>
-          <t>Old</t>
+          <t>Clinical</t>
         </is>
       </c>
       <c r="P289" t="inlineStr">
@@ -23584,7 +23630,7 @@
     </row>
     <row r="290">
       <c r="A290" t="n">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B290" t="inlineStr">
         <is>
@@ -23593,43 +23639,43 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>General Self‐Efficacy, Not Musculoskeletal Health, Was Associated With Social Isolation And Loneliness In Older Adults During The Covid‐19 Pandemic: Findings From The Hertfordshire Cohort Study</t>
+          <t>Kids Or No Kids? Life Goals In One’S 20S Predict Midlife Trajectories Of Well-Being</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s40520-023-02676-5</t>
+          <t>https://doi.org/10.1037/pag0000862</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>Hertfordshire Cohort Study</t>
+          <t>German Socio-Economic Panel (SOEP)</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>HCS</t>
+          <t>SOEP</t>
         </is>
       </c>
       <c r="G290" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>https://www.mrc.soton.ac.uk/herts/</t>
+          <t>https://www.diw.de/en/diw_01.c.791582.en/documentation_of_the_soep_studies_-_all_survey_papers.html?soep_datensatz_id[]=696367</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="J290" t="n">
-        <v>176</v>
+        <v>562</v>
       </c>
       <c r="K290" t="inlineStr">
         <is>
-          <t>CAWI</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="L290" t="inlineStr">
@@ -23639,48 +23685,43 @@
       </c>
       <c r="M290" t="inlineStr">
         <is>
-          <t>Convenience</t>
+          <t>Representative</t>
         </is>
       </c>
       <c r="N290" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>Young, Parents</t>
         </is>
       </c>
       <c r="P290" t="inlineStr">
         <is>
-          <t>DJG-6</t>
+          <t>I often feel lonely</t>
         </is>
       </c>
       <c r="Q290" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R290" t="inlineStr">
         <is>
-          <t>Yes-No</t>
+          <t>Strongly agree-Strongly disagree</t>
         </is>
       </c>
       <c r="S290" t="inlineStr">
         <is>
-          <t>DJG-6</t>
-        </is>
-      </c>
-      <c r="U290" t="inlineStr">
-        <is>
-          <t>Impossible to retrieve codebook of the survey</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="V290" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="n">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B291" t="inlineStr">
         <is>
@@ -23689,39 +23730,36 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Social Dysfunction And Neural Processing Of Emotional Valence Across Depressive And Anxiety Disorders</t>
+          <t>Cognitive Processing Speed And Loneliness In Stroke Survivors: Insights From A Large-Scale Cohort Study</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1155/2024/8564344</t>
+          <t>https://doi.org/10.1093/arclin/acae032</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>Netherlands Study of Depression and Anxiety - NESDA</t>
+          <t>1970 British Cohort Study - BCS70</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>NSDA</t>
-        </is>
-      </c>
-      <c r="G291" t="n">
-        <v>2007</v>
+          <t>BCS70</t>
+        </is>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/10.1002/mpr.256</t>
+          <t>https://cls.ucl.ac.uk/cls-studies/1970-british-cohort-study-2/</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="J291" t="n">
-        <v>200</v>
+        <v>8581</v>
       </c>
       <c r="K291" t="inlineStr">
         <is>
@@ -23735,32 +23773,32 @@
       </c>
       <c r="M291" t="inlineStr">
         <is>
-          <t>Convenience</t>
+          <t>Representative</t>
         </is>
       </c>
       <c r="N291" t="inlineStr">
         <is>
-          <t>Clinical</t>
+          <t>Adults</t>
         </is>
       </c>
       <c r="P291" t="inlineStr">
         <is>
-          <t>DJG-6</t>
+          <t>I’ve been feeling interested in other people, I’ve been feeling close to other people, I’ve been feeling loved</t>
         </is>
       </c>
       <c r="Q291" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R291" t="inlineStr">
         <is>
-          <t>Yes-No</t>
+          <t>None of the time-All of the time</t>
         </is>
       </c>
       <c r="S291" t="inlineStr">
         <is>
-          <t>DJG-6</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="U291" t="inlineStr">
@@ -23776,7 +23814,7 @@
     </row>
     <row r="292">
       <c r="A292" t="n">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B292" t="inlineStr">
         <is>
@@ -23785,43 +23823,40 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Kids Or No Kids? Life Goals In One’S 20S Predict Midlife Trajectories Of Well-Being</t>
+          <t>National Trends In Loneliness And Social Isolation In Older Adults: An Examination Of Subgroup Trends Over Three Decades In Sweden</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1037/pag0000862</t>
+          <t>https://doi.org/10.3389/fpubh.2024.1444990</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>German Socio-Economic Panel (SOEP)</t>
+          <t>Swedish Panel Study of Living Conditions of the Oldest Old -SWEOLD - 1992</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>SOEP</t>
+          <t>SWEOLD</t>
         </is>
       </c>
       <c r="G292" t="n">
-        <v>2023</v>
+        <v>1992</v>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>https://www.diw.de/en/diw_01.c.791582.en/documentation_of_the_soep_studies_-_all_survey_papers.html?soep_datensatz_id[]=696367</t>
+          <t>https://www.sweold.se/en/documentation/</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="J292" t="n">
-        <v>562</v>
+          <t>Sweden</t>
+        </is>
       </c>
       <c r="K292" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>F2F</t>
         </is>
       </c>
       <c r="L292" t="inlineStr">
@@ -23831,17 +23866,17 @@
       </c>
       <c r="M292" t="inlineStr">
         <is>
-          <t>Representative</t>
+          <t>Convenience</t>
         </is>
       </c>
       <c r="N292" t="inlineStr">
         <is>
-          <t>Young, Parents</t>
+          <t>Old</t>
         </is>
       </c>
       <c r="P292" t="inlineStr">
         <is>
-          <t>I often feel lonely</t>
+          <t>Händer det att du besväras av ensamhet?</t>
         </is>
       </c>
       <c r="Q292" t="inlineStr">
@@ -23851,12 +23886,22 @@
       </c>
       <c r="R292" t="inlineStr">
         <is>
-          <t>Strongly agree-Strongly disagree</t>
+          <t>Nästan alltid - Nästan aldrig</t>
         </is>
       </c>
       <c r="S292" t="inlineStr">
         <is>
           <t>Direct</t>
+        </is>
+      </c>
+      <c r="T292" t="inlineStr">
+        <is>
+          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation</t>
+        </is>
+      </c>
+      <c r="U292" t="inlineStr">
+        <is>
+          <t>Item wording from the published study: https://www.socialstyrelsen.se/contentassets/b8aaad069a944b99a3ca2fbc20498fa2/2026-5-10261-exempelsamling-1.pdf</t>
         </is>
       </c>
       <c r="V292" t="inlineStr">
@@ -23867,7 +23912,7 @@
     </row>
     <row r="293">
       <c r="A293" t="n">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B293" t="inlineStr">
         <is>
@@ -23876,36 +23921,36 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Cognitive Processing Speed And Loneliness In Stroke Survivors: Insights From A Large-Scale Cohort Study</t>
+          <t>National Trends In Loneliness And Social Isolation In Older Adults: An Examination Of Subgroup Trends Over Three Decades In Sweden</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1093/arclin/acae032</t>
+          <t>https://doi.org/10.3389/fpubh.2024.1444990</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>1970 British Cohort Study - BCS70</t>
+          <t>Swedish Panel Study of Living Conditions of the Oldest Old -SWEOLD - 2002</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>BCS70</t>
-        </is>
+          <t>SWEOLD</t>
+        </is>
+      </c>
+      <c r="G293" t="n">
+        <v>2002</v>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>https://cls.ucl.ac.uk/cls-studies/1970-british-cohort-study-2/</t>
+          <t>https://www.sweold.se/en/documentation/</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="J293" t="n">
-        <v>8581</v>
+          <t>Sweden</t>
+        </is>
       </c>
       <c r="K293" t="inlineStr">
         <is>
@@ -23914,53 +23959,53 @@
       </c>
       <c r="L293" t="inlineStr">
         <is>
-          <t>Panel</t>
+          <t>Repeated cross-section</t>
         </is>
       </c>
       <c r="M293" t="inlineStr">
         <is>
-          <t>Representative</t>
+          <t>Convenience</t>
         </is>
       </c>
       <c r="N293" t="inlineStr">
         <is>
-          <t>Adults</t>
+          <t>Old</t>
+        </is>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>Fråga 132</t>
         </is>
       </c>
       <c r="P293" t="inlineStr">
         <is>
-          <t>I’ve been feeling interested in other people, I’ve been feeling close to other people, I’ve been feeling loved</t>
-        </is>
-      </c>
-      <c r="Q293" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="R293" t="inlineStr">
-        <is>
-          <t>None of the time-All of the time</t>
+          <t>Händer det att Du besväras av ensamhet?</t>
         </is>
       </c>
       <c r="S293" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="T293" t="inlineStr">
+        <is>
+          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation</t>
         </is>
       </c>
       <c r="U293" t="inlineStr">
         <is>
-          <t>Impossible to retrieve codebook of the survey</t>
+          <t>Hard to understand swdish codebook</t>
         </is>
       </c>
       <c r="V293" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="n">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B294" t="inlineStr">
         <is>
@@ -23979,7 +24024,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Swedish Panel Study of Living Conditions of the Oldest Old -SWEOLD - 1992</t>
+          <t>Swedish Panel Study of Living Conditions of the Oldest Old -SWEOLD - 2004</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -23988,7 +24033,7 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>1992</v>
+        <v>2004</v>
       </c>
       <c r="H294" t="inlineStr">
         <is>
@@ -24007,7 +24052,7 @@
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t>Panel</t>
+          <t>Repeated cross-section</t>
         </is>
       </c>
       <c r="M294" t="inlineStr">
@@ -24020,9 +24065,14 @@
           <t>Old</t>
         </is>
       </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>Fråga 61</t>
+        </is>
+      </c>
       <c r="P294" t="inlineStr">
         <is>
-          <t>Händer det att du besväras av ensamhet?</t>
+          <t>Händer det att Du besväras av ensamhet?</t>
         </is>
       </c>
       <c r="Q294" t="inlineStr">
@@ -24047,7 +24097,7 @@
       </c>
       <c r="U294" t="inlineStr">
         <is>
-          <t>Item wording from the published study: https://www.socialstyrelsen.se/contentassets/b8aaad069a944b99a3ca2fbc20498fa2/2026-5-10261-exempelsamling-1.pdf</t>
+          <t>Hard to understand swdish codebook</t>
         </is>
       </c>
       <c r="V294" t="inlineStr">
@@ -24058,7 +24108,7 @@
     </row>
     <row r="295">
       <c r="A295" t="n">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B295" t="inlineStr">
         <is>
@@ -24077,7 +24127,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Swedish Panel Study of Living Conditions of the Oldest Old -SWEOLD - 2002</t>
+          <t>Swedish Panel Study of Living Conditions of the Oldest Old -SWEOLD - 2011</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -24086,7 +24136,7 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>2002</v>
+        <v>2011</v>
       </c>
       <c r="H295" t="inlineStr">
         <is>
@@ -24100,7 +24150,7 @@
       </c>
       <c r="K295" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>CATI</t>
         </is>
       </c>
       <c r="L295" t="inlineStr">
@@ -24120,12 +24170,22 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>Fråga 132</t>
+          <t>115</t>
         </is>
       </c>
       <c r="P295" t="inlineStr">
         <is>
           <t>Händer det att Du besväras av ensamhet?</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R295" t="inlineStr">
+        <is>
+          <t>Nästan alltid - Nästan aldrig</t>
         </is>
       </c>
       <c r="S295" t="inlineStr">
@@ -24151,7 +24211,7 @@
     </row>
     <row r="296">
       <c r="A296" t="n">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B296" t="inlineStr">
         <is>
@@ -24170,7 +24230,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Swedish Panel Study of Living Conditions of the Oldest Old -SWEOLD - 2004</t>
+          <t>Swedish Panel Study of Living Conditions of the Oldest Old -SWEOLD - 2014</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -24179,7 +24239,7 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>2004</v>
+        <v>2014</v>
       </c>
       <c r="H296" t="inlineStr">
         <is>
@@ -24193,7 +24253,7 @@
       </c>
       <c r="K296" t="inlineStr">
         <is>
-          <t>F2F</t>
+          <t>CATI</t>
         </is>
       </c>
       <c r="L296" t="inlineStr">
@@ -24213,7 +24273,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>Fråga 61</t>
+          <t>81</t>
         </is>
       </c>
       <c r="P296" t="inlineStr">
@@ -24254,7 +24314,7 @@
     </row>
     <row r="297">
       <c r="A297" t="n">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B297" t="inlineStr">
         <is>
@@ -24273,7 +24333,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Swedish Panel Study of Living Conditions of the Oldest Old -SWEOLD - 2011</t>
+          <t>Swedish Panel Study of Living Conditions of the Oldest Old -SWEOLD - 2021</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
@@ -24282,7 +24342,7 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>2011</v>
+        <v>2021</v>
       </c>
       <c r="H297" t="inlineStr">
         <is>
@@ -24314,14 +24374,9 @@
           <t>Old</t>
         </is>
       </c>
-      <c r="O297" t="inlineStr">
-        <is>
-          <t>115</t>
-        </is>
-      </c>
       <c r="P297" t="inlineStr">
         <is>
-          <t>Händer det att Du besväras av ensamhet?</t>
+          <t>Are you often bothered by feelings of loneliness?</t>
         </is>
       </c>
       <c r="Q297" t="inlineStr">
@@ -24331,7 +24386,7 @@
       </c>
       <c r="R297" t="inlineStr">
         <is>
-          <t>Nästan alltid - Nästan aldrig</t>
+          <t>Almost never-Nearly always</t>
         </is>
       </c>
       <c r="S297" t="inlineStr">
@@ -24346,7 +24401,7 @@
       </c>
       <c r="U297" t="inlineStr">
         <is>
-          <t>Hard to understand swdish codebook</t>
+          <t>The codebook file held for 2021 is the 2014 questionnaire; the 2021 row keeps its earlier coding.</t>
         </is>
       </c>
       <c r="V297" t="inlineStr">
@@ -24357,49 +24412,39 @@
     </row>
     <row r="298">
       <c r="A298" t="n">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Papers</t>
-        </is>
-      </c>
-      <c r="C298" t="inlineStr">
-        <is>
-          <t>National Trends In Loneliness And Social Isolation In Older Adults: An Examination Of Subgroup Trends Over Three Decades In Sweden</t>
-        </is>
-      </c>
-      <c r="D298" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.3389/fpubh.2024.1444990</t>
+          <t>Additional</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Swedish Panel Study of Living Conditions of the Oldest Old -SWEOLD - 2014</t>
+          <t>European Social Survey - ESS1 - 2002</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>SWEOLD</t>
+          <t>ESS</t>
         </is>
       </c>
       <c r="G298" t="n">
-        <v>2014</v>
+        <v>2002</v>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>https://www.sweold.se/en/documentation/</t>
+          <t>https://ess.sikt.no/en/</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Luxembourg, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
         <is>
-          <t>CATI</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="L298" t="inlineStr">
@@ -24409,47 +24454,22 @@
       </c>
       <c r="M298" t="inlineStr">
         <is>
-          <t>Convenience</t>
+          <t>Representative</t>
         </is>
       </c>
       <c r="N298" t="inlineStr">
         <is>
-          <t>Old</t>
-        </is>
-      </c>
-      <c r="O298" t="inlineStr">
-        <is>
-          <t>81</t>
-        </is>
-      </c>
-      <c r="P298" t="inlineStr">
-        <is>
-          <t>Händer det att Du besväras av ensamhet?</t>
-        </is>
-      </c>
-      <c r="Q298" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="R298" t="inlineStr">
-        <is>
-          <t>Nästan alltid - Nästan aldrig</t>
+          <t>Adults</t>
         </is>
       </c>
       <c r="S298" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>No</t>
         </is>
       </c>
       <c r="T298" t="inlineStr">
         <is>
-          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation</t>
-        </is>
-      </c>
-      <c r="U298" t="inlineStr">
-        <is>
-          <t>Hard to understand swdish codebook</t>
+          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Media use, Religion</t>
         </is>
       </c>
       <c r="V298" t="inlineStr">
@@ -24460,49 +24480,39 @@
     </row>
     <row r="299">
       <c r="A299" t="n">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Papers</t>
-        </is>
-      </c>
-      <c r="C299" t="inlineStr">
-        <is>
-          <t>National Trends In Loneliness And Social Isolation In Older Adults: An Examination Of Subgroup Trends Over Three Decades In Sweden</t>
-        </is>
-      </c>
-      <c r="D299" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.3389/fpubh.2024.1444990</t>
+          <t>Additional</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Swedish Panel Study of Living Conditions of the Oldest Old -SWEOLD - 2021</t>
+          <t>European Social Survey - ESS2 - 2004</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>SWEOLD</t>
+          <t>ESS</t>
         </is>
       </c>
       <c r="G299" t="n">
-        <v>2021</v>
+        <v>2004</v>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>https://www.sweold.se/en/documentation/</t>
+          <t>https://ess.sikt.no/en/</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Luxembourg, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Estonia, Slovakia, United Kingdom</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>CATI</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="L299" t="inlineStr">
@@ -24512,42 +24522,22 @@
       </c>
       <c r="M299" t="inlineStr">
         <is>
-          <t>Convenience</t>
+          <t>Representative</t>
         </is>
       </c>
       <c r="N299" t="inlineStr">
         <is>
-          <t>Old</t>
-        </is>
-      </c>
-      <c r="P299" t="inlineStr">
-        <is>
-          <t>Are you often bothered by feelings of loneliness?</t>
-        </is>
-      </c>
-      <c r="Q299" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="R299" t="inlineStr">
-        <is>
-          <t>Almost never-Nearly always</t>
+          <t>Adults</t>
         </is>
       </c>
       <c r="S299" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>No</t>
         </is>
       </c>
       <c r="T299" t="inlineStr">
         <is>
-          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation</t>
-        </is>
-      </c>
-      <c r="U299" t="inlineStr">
-        <is>
-          <t>The codebook file held for 2021 is the 2014 questionnaire; the 2021 row keeps its earlier coding.</t>
+          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Media use, Religion</t>
         </is>
       </c>
       <c r="V299" t="inlineStr">
@@ -24558,7 +24548,7 @@
     </row>
     <row r="300">
       <c r="A300" t="n">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B300" t="inlineStr">
         <is>
@@ -24567,7 +24557,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>European Social Survey - ESS1 - 2002</t>
+          <t>European Social Survey - ESS3 - 2006</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
@@ -24576,7 +24566,7 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>2002</v>
+        <v>2006</v>
       </c>
       <c r="H300" t="inlineStr">
         <is>
@@ -24585,7 +24575,7 @@
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Luxembourg, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia</t>
+          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Luxembourg, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Bulgaria, Cyprus, Estonia, Latvia, Romania, Slovakia, Spain, United Kingdom</t>
         </is>
       </c>
       <c r="K300" t="inlineStr">
@@ -24608,9 +24598,19 @@
           <t>Adults</t>
         </is>
       </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>E12</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>you felt lonely?</t>
+        </is>
+      </c>
       <c r="S300" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="T300" t="inlineStr">
@@ -24626,7 +24626,7 @@
     </row>
     <row r="301">
       <c r="A301" t="n">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B301" t="inlineStr">
         <is>
@@ -24635,7 +24635,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>European Social Survey - ESS2 - 2004</t>
+          <t>European Social Survey - ESS4 - 2008</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -24644,7 +24644,7 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>2004</v>
+        <v>2008</v>
       </c>
       <c r="H301" t="inlineStr">
         <is>
@@ -24653,7 +24653,7 @@
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Luxembourg, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Estonia, Slovakia, United Kingdom</t>
+          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Luxembourg, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Bulgaria, Cyprus, Estonia, Latvia, Romania, Slovakia, Spain, United Kingdom, Croatia, Lithuania</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
@@ -24694,7 +24694,7 @@
     </row>
     <row r="302">
       <c r="A302" t="n">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B302" t="inlineStr">
         <is>
@@ -24703,7 +24703,7 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>European Social Survey - ESS3 - 2006</t>
+          <t>European Social Survey - ESS5 - 2010</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
@@ -24712,7 +24712,7 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>2006</v>
+        <v>2010</v>
       </c>
       <c r="H302" t="inlineStr">
         <is>
@@ -24721,7 +24721,7 @@
       </c>
       <c r="I302" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Luxembourg, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Bulgaria, Cyprus, Estonia, Latvia, Romania, Slovakia, Spain, United Kingdom</t>
+          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Hungary, Ireland, Italy, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Estonia, Spain, United Kingdom, Lithuania</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
@@ -24746,12 +24746,22 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>E12</t>
+          <t>G71</t>
         </is>
       </c>
       <c r="P302" t="inlineStr">
         <is>
-          <t>you felt lonely?</t>
+          <t>Using this card, please tell me how much of the time during the past week you felt lonely?</t>
+        </is>
+      </c>
+      <c r="Q302" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R302" t="inlineStr">
+        <is>
+          <t>None or almost none of the time - All or almost all of the time</t>
         </is>
       </c>
       <c r="S302" t="inlineStr">
@@ -24772,7 +24782,7 @@
     </row>
     <row r="303">
       <c r="A303" t="n">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B303" t="inlineStr">
         <is>
@@ -24781,7 +24791,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>European Social Survey - ESS4 - 2008</t>
+          <t>European Social Survey - ESS7 - 2014</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
@@ -24790,7 +24800,7 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>2008</v>
+        <v>2014</v>
       </c>
       <c r="H303" t="inlineStr">
         <is>
@@ -24822,9 +24832,19 @@
           <t>Adults</t>
         </is>
       </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>E24</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t>you felt lonely?</t>
+        </is>
+      </c>
       <c r="S303" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="T303" t="inlineStr">
@@ -24840,7 +24860,7 @@
     </row>
     <row r="304">
       <c r="A304" t="n">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B304" t="inlineStr">
         <is>
@@ -24849,7 +24869,7 @@
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>European Social Survey - ESS5 - 2010</t>
+          <t>European Social Survey - ESS8 - 2016</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
@@ -24858,7 +24878,7 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>2010</v>
+        <v>2016</v>
       </c>
       <c r="H304" t="inlineStr">
         <is>
@@ -24867,7 +24887,7 @@
       </c>
       <c r="I304" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Hungary, Ireland, Italy, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Estonia, Spain, United Kingdom, Lithuania</t>
+          <t>Austria, Belgium, Estonia, Finland, France, Germany, Hungary, Ireland, Italy, Lithuania, Netherlands, Norway, Poland, Portugal, Slovenia, Spain, Sweden, United Kingdom, Czech Republic</t>
         </is>
       </c>
       <c r="K304" t="inlineStr">
@@ -24890,29 +24910,9 @@
           <t>Adults</t>
         </is>
       </c>
-      <c r="O304" t="inlineStr">
-        <is>
-          <t>G71</t>
-        </is>
-      </c>
-      <c r="P304" t="inlineStr">
-        <is>
-          <t>Using this card, please tell me how much of the time during the past week you felt lonely?</t>
-        </is>
-      </c>
-      <c r="Q304" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="R304" t="inlineStr">
-        <is>
-          <t>None or almost none of the time - All or almost all of the time</t>
-        </is>
-      </c>
       <c r="S304" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>No</t>
         </is>
       </c>
       <c r="T304" t="inlineStr">
@@ -24928,7 +24928,7 @@
     </row>
     <row r="305">
       <c r="A305" t="n">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B305" t="inlineStr">
         <is>
@@ -24937,7 +24937,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>European Social Survey - ESS7 - 2014</t>
+          <t>European Social Survey - ESS9 - 2018</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
@@ -24946,7 +24946,7 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>2014</v>
+        <v>2018</v>
       </c>
       <c r="H305" t="inlineStr">
         <is>
@@ -24955,7 +24955,7 @@
       </c>
       <c r="I305" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Luxembourg, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Bulgaria, Cyprus, Estonia, Latvia, Romania, Slovakia, Spain, United Kingdom, Croatia, Lithuania</t>
+          <t>Austria, Belgium, Bulgaria, Croatia, Cyprus, Czech Republic, Denmark, Estonia, Finland, France, Germany, Hungary, Ireland, Italy, Latvia, Lithuania, Netherlands, Norway, Poland, Portugal, Romania, Slovakia, Slovenia, Spain, Sweden, United Kingdom</t>
         </is>
       </c>
       <c r="K305" t="inlineStr">
@@ -24978,19 +24978,9 @@
           <t>Adults</t>
         </is>
       </c>
-      <c r="O305" t="inlineStr">
-        <is>
-          <t>E24</t>
-        </is>
-      </c>
-      <c r="P305" t="inlineStr">
-        <is>
-          <t>you felt lonely?</t>
-        </is>
-      </c>
       <c r="S305" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>No</t>
         </is>
       </c>
       <c r="T305" t="inlineStr">
@@ -25006,7 +24996,7 @@
     </row>
     <row r="306">
       <c r="A306" t="n">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B306" t="inlineStr">
         <is>
@@ -25015,7 +25005,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>European Social Survey - ESS8 - 2016</t>
+          <t>European Social Survey - ESS10 - 2020</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
@@ -25024,7 +25014,7 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="H306" t="inlineStr">
         <is>
@@ -25033,7 +25023,7 @@
       </c>
       <c r="I306" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Estonia, Finland, France, Germany, Hungary, Ireland, Italy, Lithuania, Netherlands, Norway, Poland, Portugal, Slovenia, Spain, Sweden, United Kingdom, Czech Republic</t>
+          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Luxembourg, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Bulgaria, Cyprus, Estonia, Latvia, Romania, Slovakia, Spain, United Kingdom, Croatia, Lithuania</t>
         </is>
       </c>
       <c r="K306" t="inlineStr">
@@ -25063,7 +25053,7 @@
       </c>
       <c r="T306" t="inlineStr">
         <is>
-          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Media use, Religion</t>
+          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Media use, Religion, COVID-19</t>
         </is>
       </c>
       <c r="V306" t="inlineStr">
@@ -25074,7 +25064,7 @@
     </row>
     <row r="307">
       <c r="A307" t="n">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B307" t="inlineStr">
         <is>
@@ -25083,7 +25073,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>European Social Survey - ESS9 - 2018</t>
+          <t>European Social Survey - ESS11 - 2023</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
@@ -25092,7 +25082,7 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="H307" t="inlineStr">
         <is>
@@ -25101,7 +25091,7 @@
       </c>
       <c r="I307" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Bulgaria, Croatia, Cyprus, Czech Republic, Denmark, Estonia, Finland, France, Germany, Hungary, Ireland, Italy, Latvia, Lithuania, Netherlands, Norway, Poland, Portugal, Romania, Slovakia, Slovenia, Spain, Sweden, United Kingdom</t>
+          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Luxembourg, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Bulgaria, Cyprus, Estonia, Latvia, Romania, Slovakia, Spain, United Kingdom, Croatia, Lithuania</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
@@ -25124,14 +25114,24 @@
           <t>Adults</t>
         </is>
       </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>D24</t>
+        </is>
+      </c>
+      <c r="P307" t="inlineStr">
+        <is>
+          <t>you felt lonely?</t>
+        </is>
+      </c>
       <c r="S307" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="T307" t="inlineStr">
         <is>
-          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Media use, Religion</t>
+          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Media use, Religion, COVID-19</t>
         </is>
       </c>
       <c r="V307" t="inlineStr">
@@ -25142,7 +25142,7 @@
     </row>
     <row r="308">
       <c r="A308" t="n">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B308" t="inlineStr">
         <is>
@@ -25151,25 +25151,25 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>European Social Survey - ESS10 - 2020</t>
+          <t>World Value Survey - WVS1 - 1984</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>ESS</t>
+          <t>WVS</t>
         </is>
       </c>
       <c r="G308" t="n">
-        <v>2020</v>
+        <v>1984</v>
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>https://ess.sikt.no/en/</t>
+          <t>https://www.worldvaluessurvey.org/WVSContents.jsp</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Luxembourg, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Bulgaria, Cyprus, Estonia, Latvia, Romania, Slovakia, Spain, United Kingdom, Croatia, Lithuania</t>
+          <t>Finland, Hungary, Sweden</t>
         </is>
       </c>
       <c r="K308" t="inlineStr">
@@ -25192,14 +25192,34 @@
           <t>Adults</t>
         </is>
       </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Question 118; </t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>Do you ever feel very lonely?; Very lonely or remote from other people</t>
+        </is>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t xml:space="preserve">; </t>
+        </is>
+      </c>
+      <c r="R308" t="inlineStr">
+        <is>
+          <t xml:space="preserve">; </t>
+        </is>
+      </c>
       <c r="S308" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="T308" t="inlineStr">
         <is>
-          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Media use, Religion, COVID-19</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion</t>
         </is>
       </c>
       <c r="V308" t="inlineStr">
@@ -25210,7 +25230,7 @@
     </row>
     <row r="309">
       <c r="A309" t="n">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B309" t="inlineStr">
         <is>
@@ -25219,25 +25239,25 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>European Social Survey - ESS11 - 2023</t>
+          <t>World Value Survey - WVS2 - 1994</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>ESS</t>
+          <t>WVS</t>
         </is>
       </c>
       <c r="G309" t="n">
-        <v>2023</v>
+        <v>1994</v>
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>https://ess.sikt.no/en/</t>
+          <t>https://www.worldvaluessurvey.org/WVSContents.jsp</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Czech Republic, Denmark, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Luxembourg, Netherlands, Norway, Poland, Portugal, Sweden, Slovenia, Bulgaria, Cyprus, Estonia, Latvia, Romania, Slovakia, Spain, United Kingdom, Croatia, Lithuania</t>
+          <t>Finland, Hungary, Sweden, Czech Republic, Poland, Slovakia, Spain</t>
         </is>
       </c>
       <c r="K309" t="inlineStr">
@@ -25262,12 +25282,12 @@
       </c>
       <c r="O309" t="inlineStr">
         <is>
-          <t>D24</t>
+          <t>V 87</t>
         </is>
       </c>
       <c r="P309" t="inlineStr">
         <is>
-          <t>you felt lonely?</t>
+          <t>Very lonely or remote from other people</t>
         </is>
       </c>
       <c r="S309" t="inlineStr">
@@ -25277,7 +25297,7 @@
       </c>
       <c r="T309" t="inlineStr">
         <is>
-          <t>Health and health behaviours, Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Media use, Religion, COVID-19</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion</t>
         </is>
       </c>
       <c r="V309" t="inlineStr">
@@ -25288,7 +25308,7 @@
     </row>
     <row r="310">
       <c r="A310" t="n">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B310" t="inlineStr">
         <is>
@@ -25297,7 +25317,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>World Value Survey - WVS1 - 1984</t>
+          <t>World Value Survey - WVS3 - 1998</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
@@ -25306,7 +25326,7 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>1984</v>
+        <v>1998</v>
       </c>
       <c r="H310" t="inlineStr">
         <is>
@@ -25315,7 +25335,7 @@
       </c>
       <c r="I310" t="inlineStr">
         <is>
-          <t>Finland, Hungary, Sweden</t>
+          <t>Finland, Hungary, Sweden, Czech Republic, Poland, Slovakia, Spain, Bulgaria, Croatia, Estonia, Germany, Latvia, Lithuania, Norway, Romania, Slovenia, United Kingdom</t>
         </is>
       </c>
       <c r="K310" t="inlineStr">
@@ -25338,34 +25358,14 @@
           <t>Adults</t>
         </is>
       </c>
-      <c r="O310" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Question 118; </t>
-        </is>
-      </c>
-      <c r="P310" t="inlineStr">
-        <is>
-          <t>Do you ever feel very lonely?; Very lonely or remote from other people</t>
-        </is>
-      </c>
-      <c r="Q310" t="inlineStr">
-        <is>
-          <t xml:space="preserve">; </t>
-        </is>
-      </c>
-      <c r="R310" t="inlineStr">
-        <is>
-          <t xml:space="preserve">; </t>
-        </is>
-      </c>
       <c r="S310" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>No</t>
         </is>
       </c>
       <c r="T310" t="inlineStr">
         <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Media use</t>
         </is>
       </c>
       <c r="V310" t="inlineStr">
@@ -25376,7 +25376,7 @@
     </row>
     <row r="311">
       <c r="A311" t="n">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B311" t="inlineStr">
         <is>
@@ -25385,7 +25385,7 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>World Value Survey - WVS2 - 1994</t>
+          <t>World Value Survey - WVS4 - 2004</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
@@ -25394,7 +25394,7 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>1994</v>
+        <v>2004</v>
       </c>
       <c r="H311" t="inlineStr">
         <is>
@@ -25403,7 +25403,7 @@
       </c>
       <c r="I311" t="inlineStr">
         <is>
-          <t>Finland, Hungary, Sweden, Czech Republic, Poland, Slovakia, Spain</t>
+          <t>Spain, Sweden</t>
         </is>
       </c>
       <c r="K311" t="inlineStr">
@@ -25426,24 +25426,14 @@
           <t>Adults</t>
         </is>
       </c>
-      <c r="O311" t="inlineStr">
-        <is>
-          <t>V 87</t>
-        </is>
-      </c>
-      <c r="P311" t="inlineStr">
-        <is>
-          <t>Very lonely or remote from other people</t>
-        </is>
-      </c>
       <c r="S311" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>No</t>
         </is>
       </c>
       <c r="T311" t="inlineStr">
         <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Media use</t>
         </is>
       </c>
       <c r="V311" t="inlineStr">
@@ -25454,7 +25444,7 @@
     </row>
     <row r="312">
       <c r="A312" t="n">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B312" t="inlineStr">
         <is>
@@ -25463,7 +25453,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>World Value Survey - WVS3 - 1998</t>
+          <t>World Value Survey - WVS5 - 2009</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
@@ -25472,7 +25462,7 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>1998</v>
+        <v>2009</v>
       </c>
       <c r="H312" t="inlineStr">
         <is>
@@ -25481,7 +25471,7 @@
       </c>
       <c r="I312" t="inlineStr">
         <is>
-          <t>Finland, Hungary, Sweden, Czech Republic, Poland, Slovakia, Spain, Bulgaria, Croatia, Estonia, Germany, Latvia, Lithuania, Norway, Romania, Slovenia, United Kingdom</t>
+          <t>Bulgaria, Cyprus, Finland, France, Germany, Hungary, Italy, Netherlands, Norway, Poland, Romania, Slovenia, Spain, Sweden, United Kingdom</t>
         </is>
       </c>
       <c r="K312" t="inlineStr">
@@ -25511,7 +25501,7 @@
       </c>
       <c r="T312" t="inlineStr">
         <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Media use</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Media use, Online activities</t>
         </is>
       </c>
       <c r="V312" t="inlineStr">
@@ -25522,7 +25512,7 @@
     </row>
     <row r="313">
       <c r="A313" t="n">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B313" t="inlineStr">
         <is>
@@ -25531,7 +25521,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>World Value Survey - WVS4 - 2004</t>
+          <t>World Value Survey - WVS6 - 2014</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
@@ -25540,7 +25530,7 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>2004</v>
+        <v>2014</v>
       </c>
       <c r="H313" t="inlineStr">
         <is>
@@ -25549,7 +25539,7 @@
       </c>
       <c r="I313" t="inlineStr">
         <is>
-          <t>Spain, Sweden</t>
+          <t>Cyprus, Estonia, Germany, Netherlands, Poland, Romania, Slovenia, Spain, Sweden</t>
         </is>
       </c>
       <c r="K313" t="inlineStr">
@@ -25579,7 +25569,7 @@
       </c>
       <c r="T313" t="inlineStr">
         <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Media use</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Media use, Online activities</t>
         </is>
       </c>
       <c r="V313" t="inlineStr">
@@ -25590,7 +25580,7 @@
     </row>
     <row r="314">
       <c r="A314" t="n">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B314" t="inlineStr">
         <is>
@@ -25599,7 +25589,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>World Value Survey - WVS5 - 2009</t>
+          <t>World Value Survey - WVS7 - 2022</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -25608,7 +25598,7 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>2009</v>
+        <v>2022</v>
       </c>
       <c r="H314" t="inlineStr">
         <is>
@@ -25617,7 +25607,7 @@
       </c>
       <c r="I314" t="inlineStr">
         <is>
-          <t>Bulgaria, Cyprus, Finland, France, Germany, Hungary, Italy, Netherlands, Norway, Poland, Romania, Slovenia, Spain, Sweden, United Kingdom</t>
+          <t>Austria, Bulgaria, Croatia, Czech Republic, Denmark, Estonia, Finland, France, Germany, Greece, Hungary, Italy, Latvia, Lithuania, Netherlands, Poland, Portugal, Romania, Slovakia, Slovenia, Spain, Sweden, United Kingdom, Norway</t>
         </is>
       </c>
       <c r="K314" t="inlineStr">
@@ -25658,7 +25648,7 @@
     </row>
     <row r="315">
       <c r="A315" t="n">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B315" t="inlineStr">
         <is>
@@ -25667,25 +25657,25 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>World Value Survey - WVS6 - 2014</t>
+          <t>European Values Study - EVS1 - 1981</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>WVS</t>
+          <t>EVS</t>
         </is>
       </c>
       <c r="G315" t="n">
-        <v>2014</v>
+        <v>1981</v>
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>https://www.worldvaluessurvey.org/WVSContents.jsp</t>
+          <t>https://search.gesis.org/?source=%7B%22query%22%3A%7B%22bool%22%3A%7B%22must%22%3A%7B%22match_all%22%3A%7B%7D%7D%2C%22filter%22%3A%5B%7B%22term%22%3A%7B%22type%22%3A%22research_data%22%7D%7D%2C%7B%22term%22%3A%7B%22study_group_en.keyword%22%3A%22EVS%201981%22%7D%7D%5D%7D%7D%7D&amp;lang=en</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
         <is>
-          <t>Cyprus, Estonia, Germany, Netherlands, Poland, Romania, Slovenia, Spain, Sweden</t>
+          <t>Belgium, Denmark, France, Germany, United Kingdom, Ireland, Italy, Malta, Netherlands, Norway, Spain, Sweden</t>
         </is>
       </c>
       <c r="K315" t="inlineStr">
@@ -25708,14 +25698,34 @@
           <t>Adults</t>
         </is>
       </c>
+      <c r="O315" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Question 118; </t>
+        </is>
+      </c>
+      <c r="P315" t="inlineStr">
+        <is>
+          <t>Do you ever feel very lonely?; Very lonely or remote from other people</t>
+        </is>
+      </c>
+      <c r="Q315" t="inlineStr">
+        <is>
+          <t xml:space="preserve">; </t>
+        </is>
+      </c>
+      <c r="R315" t="inlineStr">
+        <is>
+          <t xml:space="preserve">; </t>
+        </is>
+      </c>
       <c r="S315" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="T315" t="inlineStr">
         <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Media use, Online activities</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion</t>
         </is>
       </c>
       <c r="V315" t="inlineStr">
@@ -25726,7 +25736,7 @@
     </row>
     <row r="316">
       <c r="A316" t="n">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B316" t="inlineStr">
         <is>
@@ -25735,25 +25745,25 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>World Value Survey - WVS7 - 2022</t>
+          <t>European Values Study - EVS2 - 1990</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>WVS</t>
+          <t>EVS</t>
         </is>
       </c>
       <c r="G316" t="n">
-        <v>2022</v>
+        <v>1990</v>
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>https://www.worldvaluessurvey.org/WVSContents.jsp</t>
+          <t>https://search.gesis.org/research_data/ZA4460?doi=10.4232/1.10790</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
         <is>
-          <t>Austria, Bulgaria, Croatia, Czech Republic, Denmark, Estonia, Finland, France, Germany, Greece, Hungary, Italy, Latvia, Lithuania, Netherlands, Poland, Portugal, Romania, Slovakia, Slovenia, Spain, Sweden, United Kingdom, Norway</t>
+          <t>Austria, Belgium, Bulgaria, Czech Republic, Denmark, Estonia, Finland, France, Germany, Hungary, Ireland, Italy, Latvia, Lithuania, Malta, Netherlands, Poland, Portugal, Romania, Slovenia, Spain, Sweden, United Kingdom, Norway</t>
         </is>
       </c>
       <c r="K316" t="inlineStr">
@@ -25776,14 +25786,19 @@
           <t>Adults</t>
         </is>
       </c>
+      <c r="P316" t="inlineStr">
+        <is>
+          <t>Very lonely or remote from other people</t>
+        </is>
+      </c>
       <c r="S316" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="T316" t="inlineStr">
         <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Media use, Online activities</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion</t>
         </is>
       </c>
       <c r="V316" t="inlineStr">
@@ -25794,7 +25809,7 @@
     </row>
     <row r="317">
       <c r="A317" t="n">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B317" t="inlineStr">
         <is>
@@ -25803,7 +25818,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>European Values Study - EVS1 - 1981</t>
+          <t>European Values Study - EVS3 - 1999</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
@@ -25812,16 +25827,16 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>1981</v>
+        <v>1999</v>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>https://search.gesis.org/?source=%7B%22query%22%3A%7B%22bool%22%3A%7B%22must%22%3A%7B%22match_all%22%3A%7B%7D%7D%2C%22filter%22%3A%5B%7B%22term%22%3A%7B%22type%22%3A%22research_data%22%7D%7D%2C%7B%22term%22%3A%7B%22study_group_en.keyword%22%3A%22EVS%201981%22%7D%7D%5D%7D%7D%7D&amp;lang=en</t>
+          <t>https://search.gesis.org/research_data/ZA3811?doi=10.4232/1.10789</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
         <is>
-          <t>Belgium, Denmark, France, Germany, United Kingdom, Ireland, Italy, Malta, Netherlands, Norway, Spain, Sweden</t>
+          <t>Austria, Belgium, Bulgaria, Czech Republic, Denmark, Estonia, Finland, France, Germany, Hungary, Ireland, Italy, Latvia, Lithuania, Malta, Netherlands, Poland, Portugal, Romania, Slovenia, Spain, Sweden, United Kingdom, Norway, Croatia, Greece, Luxembourg, Slovakia</t>
         </is>
       </c>
       <c r="K317" t="inlineStr">
@@ -25844,34 +25859,14 @@
           <t>Adults</t>
         </is>
       </c>
-      <c r="O317" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Question 118; </t>
-        </is>
-      </c>
-      <c r="P317" t="inlineStr">
-        <is>
-          <t>Do you ever feel very lonely?; Very lonely or remote from other people</t>
-        </is>
-      </c>
-      <c r="Q317" t="inlineStr">
-        <is>
-          <t xml:space="preserve">; </t>
-        </is>
-      </c>
-      <c r="R317" t="inlineStr">
-        <is>
-          <t xml:space="preserve">; </t>
-        </is>
-      </c>
       <c r="S317" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>No</t>
         </is>
       </c>
       <c r="T317" t="inlineStr">
         <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Media use</t>
         </is>
       </c>
       <c r="V317" t="inlineStr">
@@ -25882,7 +25877,7 @@
     </row>
     <row r="318">
       <c r="A318" t="n">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B318" t="inlineStr">
         <is>
@@ -25891,7 +25886,7 @@
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>European Values Study - EVS2 - 1990</t>
+          <t>European Values Study - EVS4 - 2008</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
@@ -25900,16 +25895,16 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>1990</v>
+        <v>2008</v>
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>https://search.gesis.org/research_data/ZA4460?doi=10.4232/1.10790</t>
+          <t>https://search.gesis.org/research_data/ZA4800</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Bulgaria, Czech Republic, Denmark, Estonia, Finland, France, Germany, Hungary, Ireland, Italy, Latvia, Lithuania, Malta, Netherlands, Poland, Portugal, Romania, Slovenia, Spain, Sweden, United Kingdom, Norway</t>
+          <t>Austria, Belgium, Bulgaria, Czech Republic, Denmark, Estonia, Finland, France, Germany, Hungary, Ireland, Italy, Latvia, Lithuania, Malta, Netherlands, Poland, Portugal, Romania, Slovenia, Spain, Sweden, United Kingdom, Norway, Croatia, Greece, Luxembourg, Slovakia, Cyprus</t>
         </is>
       </c>
       <c r="K318" t="inlineStr">
@@ -25932,19 +25927,14 @@
           <t>Adults</t>
         </is>
       </c>
-      <c r="P318" t="inlineStr">
-        <is>
-          <t>Very lonely or remote from other people</t>
-        </is>
-      </c>
       <c r="S318" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>No</t>
         </is>
       </c>
       <c r="T318" t="inlineStr">
         <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Media use</t>
         </is>
       </c>
       <c r="V318" t="inlineStr">
@@ -25955,7 +25945,7 @@
     </row>
     <row r="319">
       <c r="A319" t="n">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B319" t="inlineStr">
         <is>
@@ -25964,7 +25954,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>European Values Study - EVS3 - 1999</t>
+          <t>European Values Study - EVS5 - 2017</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
@@ -25973,11 +25963,11 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>1999</v>
+        <v>2017</v>
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>https://search.gesis.org/research_data/ZA3811?doi=10.4232/1.10789</t>
+          <t>https://search.gesis.org/research_data/ZA7500</t>
         </is>
       </c>
       <c r="I319" t="inlineStr">
@@ -25987,7 +25977,7 @@
       </c>
       <c r="K319" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>CAWI</t>
         </is>
       </c>
       <c r="L319" t="inlineStr">
@@ -26012,7 +26002,7 @@
       </c>
       <c r="T319" t="inlineStr">
         <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Media use</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Online activities, Media use</t>
         </is>
       </c>
       <c r="V319" t="inlineStr">
@@ -26023,7 +26013,7 @@
     </row>
     <row r="320">
       <c r="A320" t="n">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B320" t="inlineStr">
         <is>
@@ -26032,35 +26022,38 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>European Values Study - EVS4 - 2008</t>
+          <t>EU Loneliness Survey - EU4 sample</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>EVS</t>
+          <t>EULS4</t>
         </is>
       </c>
       <c r="G320" t="n">
-        <v>2008</v>
+        <v>2022</v>
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>https://search.gesis.org/research_data/ZA4800</t>
+          <t>https://data.jrc.ec.europa.eu/dataset/82e60986-9987-4610-ab4a-84f0f5a9193b</t>
         </is>
       </c>
       <c r="I320" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Bulgaria, Czech Republic, Denmark, Estonia, Finland, France, Germany, Hungary, Ireland, Italy, Latvia, Lithuania, Malta, Netherlands, Poland, Portugal, Romania, Slovenia, Spain, Sweden, United Kingdom, Norway, Croatia, Greece, Luxembourg, Slovakia, Cyprus</t>
-        </is>
+          <t>France, Italy, Poland, Sweden</t>
+        </is>
+      </c>
+      <c r="J320" t="n">
+        <v>4029</v>
       </c>
       <c r="K320" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>CAWI</t>
         </is>
       </c>
       <c r="L320" t="inlineStr">
         <is>
-          <t>Repeated cross-section</t>
+          <t>Cross-section</t>
         </is>
       </c>
       <c r="M320" t="inlineStr">
@@ -26073,14 +26066,34 @@
           <t>Adults</t>
         </is>
       </c>
+      <c r="O320" t="inlineStr">
+        <is>
+          <t>loneliness_djg; loneliness_djg; loneliness_djg; loneliness_djg; loneliness_djg; loneliness_djg; loneliness_ucla; loneliness_ucla; loneliness_ucla; loneliness_direct; loneliness_intensity</t>
+        </is>
+      </c>
+      <c r="P320" t="inlineStr">
+        <is>
+          <t>Please indicate for each of the statements, the extent to which they apply to your situation and the I experience a general sense of emptiness; I miss having people around; I often feel rejected; There are plenty of people I can rely on when I have; There are many people I can trust completely; There are enough people that I feel close to; Please indicate how often you feel each of the following: Feel that you lack companionship; Feel left out; Feel isolated from others; How much of the time, during the past 4 weeks, have you been feeling lonely?; How intense was this feeling of loneliness?</t>
+        </is>
+      </c>
+      <c r="Q320" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3; 3; 3; 3; 3; 3; 3; 3; 3; 5; </t>
+        </is>
+      </c>
+      <c r="R320" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes - No; Yes - No; Yes - No; Yes - No; Yes - No; Yes - No; Hardly ever or never - Often; Hardly ever or never - Often; Hardly ever or never - Often; All of the time - None of the time; </t>
+        </is>
+      </c>
       <c r="S320" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>UCLA-3, DJG-6, Direct</t>
         </is>
       </c>
       <c r="T320" t="inlineStr">
         <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Media use</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Religion, COVID-19, Online activities, Media use</t>
         </is>
       </c>
       <c r="V320" t="inlineStr">
@@ -26091,7 +26104,7 @@
     </row>
     <row r="321">
       <c r="A321" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B321" t="inlineStr">
         <is>
@@ -26100,26 +26113,29 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>European Values Study - EVS5 - 2017</t>
+          <t>EU Loneliness Survey - EU4 sample</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>EVS</t>
+          <t>EULS27</t>
         </is>
       </c>
       <c r="G321" t="n">
-        <v>2017</v>
+        <v>2022</v>
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>https://search.gesis.org/research_data/ZA7500</t>
+          <t>https://data.jrc.ec.europa.eu/dataset/82e60986-9987-4610-ab4a-84f0f5a9193b</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
         <is>
-          <t>Austria, Belgium, Bulgaria, Czech Republic, Denmark, Estonia, Finland, France, Germany, Hungary, Ireland, Italy, Latvia, Lithuania, Malta, Netherlands, Poland, Portugal, Romania, Slovenia, Spain, Sweden, United Kingdom, Norway, Croatia, Greece, Luxembourg, Slovakia</t>
-        </is>
+          <t>Austria, Belgium, Bulgaria, Croatia, Cyprus, Czech Republic, Denmark, Estonia, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Latvia, Lithuania, Luxembourg, Malta, Netherlands, Poland, Portugal, Romania, Slovakia, Slovenia, Spain, Sweden</t>
+        </is>
+      </c>
+      <c r="J321" t="n">
+        <v>25646</v>
       </c>
       <c r="K321" t="inlineStr">
         <is>
@@ -26128,12 +26144,12 @@
       </c>
       <c r="L321" t="inlineStr">
         <is>
-          <t>Repeated cross-section</t>
+          <t>Cross-section</t>
         </is>
       </c>
       <c r="M321" t="inlineStr">
         <is>
-          <t>Representative</t>
+          <t>Convenience</t>
         </is>
       </c>
       <c r="N321" t="inlineStr">
@@ -26141,199 +26157,37 @@
           <t>Adults</t>
         </is>
       </c>
+      <c r="O321" t="inlineStr">
+        <is>
+          <t>loneliness_djg; loneliness_djg; loneliness_djg; loneliness_djg; loneliness_djg; loneliness_djg; loneliness_ucla; loneliness_ucla; loneliness_ucla; loneliness_direct; loneliness_intensity</t>
+        </is>
+      </c>
+      <c r="P321" t="inlineStr">
+        <is>
+          <t>Please indicate for each of the statements, the extent to which they apply to your situation and the I experience a general sense of emptiness; I miss having people around; I often feel rejected; There are plenty of people I can rely on when I have; There are many people I can trust completely; There are enough people that I feel close to; Please indicate how often you feel each of the following: Feel that you lack companionship; Feel left out; Feel isolated from others; How much of the time, during the past 4 weeks, have you been feeling lonely?; How intense was this feeling of loneliness?</t>
+        </is>
+      </c>
+      <c r="Q321" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3; 3; 3; 3; 3; 3; 3; 3; 3; 5; </t>
+        </is>
+      </c>
+      <c r="R321" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes - No; Yes - No; Yes - No; Yes - No; Yes - No; Yes - No; Hardly ever or never - Often; Hardly ever or never - Often; Hardly ever or never - Often; All of the time - None of the time; </t>
+        </is>
+      </c>
       <c r="S321" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>UCLA-3, DJG-6, Direct</t>
         </is>
       </c>
       <c r="T321" t="inlineStr">
         <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Politics and values, Religion, Online activities, Media use</t>
+          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Religion, COVID-19, Online activities, Media use</t>
         </is>
       </c>
       <c r="V321" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="n">
-        <v>321</v>
-      </c>
-      <c r="B322" t="inlineStr">
-        <is>
-          <t>Additional</t>
-        </is>
-      </c>
-      <c r="E322" t="inlineStr">
-        <is>
-          <t>EU Loneliness Survey - EU4 sample</t>
-        </is>
-      </c>
-      <c r="F322" t="inlineStr">
-        <is>
-          <t>EULS4</t>
-        </is>
-      </c>
-      <c r="G322" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H322" t="inlineStr">
-        <is>
-          <t>https://data.jrc.ec.europa.eu/dataset/82e60986-9987-4610-ab4a-84f0f5a9193b</t>
-        </is>
-      </c>
-      <c r="I322" t="inlineStr">
-        <is>
-          <t>France, Italy, Poland, Sweden</t>
-        </is>
-      </c>
-      <c r="J322" t="n">
-        <v>4029</v>
-      </c>
-      <c r="K322" t="inlineStr">
-        <is>
-          <t>CAWI</t>
-        </is>
-      </c>
-      <c r="L322" t="inlineStr">
-        <is>
-          <t>Cross-section</t>
-        </is>
-      </c>
-      <c r="M322" t="inlineStr">
-        <is>
-          <t>Representative</t>
-        </is>
-      </c>
-      <c r="N322" t="inlineStr">
-        <is>
-          <t>Adults</t>
-        </is>
-      </c>
-      <c r="O322" t="inlineStr">
-        <is>
-          <t>loneliness_djg; loneliness_djg; loneliness_djg; loneliness_djg; loneliness_djg; loneliness_djg; loneliness_ucla; loneliness_ucla; loneliness_ucla; loneliness_direct; loneliness_intensity</t>
-        </is>
-      </c>
-      <c r="P322" t="inlineStr">
-        <is>
-          <t>Please indicate for each of the statements, the extent to which they apply to your situation and the I experience a general sense of emptiness; I miss having people around; I often feel rejected; There are plenty of people I can rely on when I have; There are many people I can trust completely; There are enough people that I feel close to; Please indicate how often you feel each of the following: Feel that you lack companionship; Feel left out; Feel isolated from others; How much of the time, during the past 4 weeks, have you been feeling lonely?; How intense was this feeling of loneliness?</t>
-        </is>
-      </c>
-      <c r="Q322" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3; 3; 3; 3; 3; 3; 3; 3; 3; 5; </t>
-        </is>
-      </c>
-      <c r="R322" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes - No; Yes - No; Yes - No; Yes - No; Yes - No; Yes - No; Hardly ever or never - Often; Hardly ever or never - Often; Hardly ever or never - Often; All of the time - None of the time; </t>
-        </is>
-      </c>
-      <c r="S322" t="inlineStr">
-        <is>
-          <t>UCLA-3, DJG-6, Direct</t>
-        </is>
-      </c>
-      <c r="T322" t="inlineStr">
-        <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Religion, COVID-19, Online activities, Media use</t>
-        </is>
-      </c>
-      <c r="V322" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="n">
-        <v>322</v>
-      </c>
-      <c r="B323" t="inlineStr">
-        <is>
-          <t>Additional</t>
-        </is>
-      </c>
-      <c r="E323" t="inlineStr">
-        <is>
-          <t>EU Loneliness Survey - EU4 sample</t>
-        </is>
-      </c>
-      <c r="F323" t="inlineStr">
-        <is>
-          <t>EULS27</t>
-        </is>
-      </c>
-      <c r="G323" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H323" t="inlineStr">
-        <is>
-          <t>https://data.jrc.ec.europa.eu/dataset/82e60986-9987-4610-ab4a-84f0f5a9193b</t>
-        </is>
-      </c>
-      <c r="I323" t="inlineStr">
-        <is>
-          <t>Austria, Belgium, Bulgaria, Croatia, Cyprus, Czech Republic, Denmark, Estonia, Finland, France, Germany, Greece, Hungary, Ireland, Italy, Latvia, Lithuania, Luxembourg, Malta, Netherlands, Poland, Portugal, Romania, Slovakia, Slovenia, Spain, Sweden</t>
-        </is>
-      </c>
-      <c r="J323" t="n">
-        <v>25646</v>
-      </c>
-      <c r="K323" t="inlineStr">
-        <is>
-          <t>CAWI</t>
-        </is>
-      </c>
-      <c r="L323" t="inlineStr">
-        <is>
-          <t>Cross-section</t>
-        </is>
-      </c>
-      <c r="M323" t="inlineStr">
-        <is>
-          <t>Convenience</t>
-        </is>
-      </c>
-      <c r="N323" t="inlineStr">
-        <is>
-          <t>Adults</t>
-        </is>
-      </c>
-      <c r="O323" t="inlineStr">
-        <is>
-          <t>loneliness_djg; loneliness_djg; loneliness_djg; loneliness_djg; loneliness_djg; loneliness_djg; loneliness_ucla; loneliness_ucla; loneliness_ucla; loneliness_direct; loneliness_intensity</t>
-        </is>
-      </c>
-      <c r="P323" t="inlineStr">
-        <is>
-          <t>Please indicate for each of the statements, the extent to which they apply to your situation and the I experience a general sense of emptiness; I miss having people around; I often feel rejected; There are plenty of people I can rely on when I have; There are many people I can trust completely; There are enough people that I feel close to; Please indicate how often you feel each of the following: Feel that you lack companionship; Feel left out; Feel isolated from others; How much of the time, during the past 4 weeks, have you been feeling lonely?; How intense was this feeling of loneliness?</t>
-        </is>
-      </c>
-      <c r="Q323" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3; 3; 3; 3; 3; 3; 3; 3; 3; 5; </t>
-        </is>
-      </c>
-      <c r="R323" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes - No; Yes - No; Yes - No; Yes - No; Yes - No; Yes - No; Hardly ever or never - Often; Hardly ever or never - Often; Hardly ever or never - Often; All of the time - None of the time; </t>
-        </is>
-      </c>
-      <c r="S323" t="inlineStr">
-        <is>
-          <t>UCLA-3, DJG-6, Direct</t>
-        </is>
-      </c>
-      <c r="T323" t="inlineStr">
-        <is>
-          <t>Mental health and wellbeing, Social relations and social support, Demographics and housing composition, Socioeconomic conditions and employment, Housing and living conditions, Community and social participation, Politics and values, Religion, COVID-19, Online activities, Media use</t>
-        </is>
-      </c>
-      <c r="V323" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>